<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-28 (sentiment: 4.17)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J488"/>
+  <dimension ref="A1:J489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16050,7 +16050,7 @@
         <v>20.11</v>
       </c>
       <c r="E488" t="n">
-        <v>7.74</v>
+        <v>6.82</v>
       </c>
       <c r="F488" t="n">
         <v>0.6</v>
@@ -16062,10 +16062,34 @@
         <v>10.91</v>
       </c>
       <c r="I488" t="n">
-        <v>7.34</v>
+        <v>3.37</v>
       </c>
       <c r="J488" t="n">
-        <v>20.93</v>
+        <v>19.94</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="n">
+        <v>46293.66666666666</v>
+      </c>
+      <c r="B489" t="inlineStr"/>
+      <c r="C489" t="inlineStr"/>
+      <c r="D489" t="n">
+        <v>16.13</v>
+      </c>
+      <c r="E489" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="F489" t="inlineStr"/>
+      <c r="G489" t="inlineStr"/>
+      <c r="H489" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="I489" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J489" t="n">
+        <v>4.17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-29 (sentiment: 39.48)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J489"/>
+  <dimension ref="A1:J490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16078,7 +16078,7 @@
         <v>16.13</v>
       </c>
       <c r="E489" t="n">
-        <v>6.61</v>
+        <v>6.39</v>
       </c>
       <c r="F489" t="inlineStr"/>
       <c r="G489" t="inlineStr"/>
@@ -16086,10 +16086,34 @@
         <v>6.94</v>
       </c>
       <c r="I489" t="n">
-        <v>1.39</v>
+        <v>0.2</v>
       </c>
       <c r="J489" t="n">
-        <v>4.17</v>
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="n">
+        <v>46294.66666666666</v>
+      </c>
+      <c r="B490" t="inlineStr"/>
+      <c r="C490" t="inlineStr"/>
+      <c r="D490" t="n">
+        <v>62.32</v>
+      </c>
+      <c r="E490" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="F490" t="inlineStr"/>
+      <c r="G490" t="inlineStr"/>
+      <c r="H490" t="n">
+        <v>71.23</v>
+      </c>
+      <c r="I490" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="J490" t="n">
+        <v>39.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-30 (sentiment: 29.76)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J490"/>
+  <dimension ref="A1:J491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16072,16 +16072,24 @@
       <c r="A489" s="2" t="n">
         <v>46293.66666666666</v>
       </c>
-      <c r="B489" t="inlineStr"/>
-      <c r="C489" t="inlineStr"/>
+      <c r="B489" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="C489" t="n">
+        <v>44.24</v>
+      </c>
       <c r="D489" t="n">
         <v>16.13</v>
       </c>
       <c r="E489" t="n">
         <v>6.39</v>
       </c>
-      <c r="F489" t="inlineStr"/>
-      <c r="G489" t="inlineStr"/>
+      <c r="F489" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="G489" t="n">
+        <v>72.02</v>
+      </c>
       <c r="H489" t="n">
         <v>6.94</v>
       </c>
@@ -16089,31 +16097,71 @@
         <v>0.2</v>
       </c>
       <c r="J489" t="n">
-        <v>3.57</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n">
         <v>46294.66666666666</v>
       </c>
-      <c r="B490" t="inlineStr"/>
-      <c r="C490" t="inlineStr"/>
+      <c r="B490" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="C490" t="n">
+        <v>41.05</v>
+      </c>
       <c r="D490" t="n">
         <v>62.32</v>
       </c>
       <c r="E490" t="n">
-        <v>7.72</v>
-      </c>
-      <c r="F490" t="inlineStr"/>
-      <c r="G490" t="inlineStr"/>
+        <v>6.97</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G490" t="n">
+        <v>58.53</v>
+      </c>
       <c r="H490" t="n">
         <v>71.23</v>
       </c>
       <c r="I490" t="n">
-        <v>7.74</v>
+        <v>4.56</v>
       </c>
       <c r="J490" t="n">
-        <v>39.48</v>
+        <v>33.63</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="B491" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="C491" t="n">
+        <v>42.73</v>
+      </c>
+      <c r="D491" t="n">
+        <v>46.06</v>
+      </c>
+      <c r="E491" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G491" t="n">
+        <v>64.48</v>
+      </c>
+      <c r="H491" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="I491" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="J491" t="n">
+        <v>29.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-08 (sentiment: 24.01)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J491"/>
+  <dimension ref="A1:J492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16146,7 +16146,7 @@
         <v>46.06</v>
       </c>
       <c r="E491" t="n">
-        <v>6.82</v>
+        <v>6.27</v>
       </c>
       <c r="F491" t="n">
         <v>0.2</v>
@@ -16158,10 +16158,42 @@
         <v>50.6</v>
       </c>
       <c r="I491" t="n">
-        <v>3.77</v>
+        <v>0.2</v>
       </c>
       <c r="J491" t="n">
-        <v>29.76</v>
+        <v>28.87</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="n">
+        <v>46303.66666666666</v>
+      </c>
+      <c r="B492" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="C492" t="n">
+        <v>43.07</v>
+      </c>
+      <c r="D492" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="E492" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="F492" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="G492" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="H492" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I492" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J492" t="n">
+        <v>24.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-09 (sentiment: 35.02)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J492"/>
+  <dimension ref="A1:J493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16178,7 +16178,7 @@
         <v>30.48</v>
       </c>
       <c r="E492" t="n">
-        <v>5.38</v>
+        <v>6.57</v>
       </c>
       <c r="F492" t="n">
         <v>2.18</v>
@@ -16190,10 +16190,42 @@
         <v>27.58</v>
       </c>
       <c r="I492" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J492" t="n">
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="B493" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="C493" t="n">
+        <v>41.53</v>
+      </c>
+      <c r="D493" t="n">
+        <v>59.15</v>
+      </c>
+      <c r="E493" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="F493" t="n">
+        <v>14.09</v>
+      </c>
+      <c r="G493" t="n">
+        <v>59.72</v>
+      </c>
+      <c r="H493" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="I493" t="n">
         <v>0.2</v>
       </c>
-      <c r="J492" t="n">
-        <v>24.01</v>
+      <c r="J493" t="n">
+        <v>35.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-12 (sentiment: 18.85)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J493"/>
+  <dimension ref="A1:J494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16210,7 +16210,7 @@
         <v>59.15</v>
       </c>
       <c r="E493" t="n">
-        <v>5.78</v>
+        <v>6.24</v>
       </c>
       <c r="F493" t="n">
         <v>14.09</v>
@@ -16226,6 +16226,38 @@
       </c>
       <c r="J493" t="n">
         <v>35.02</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="B494" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="C494" t="n">
+        <v>40.04</v>
+      </c>
+      <c r="D494" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="E494" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="F494" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G494" t="n">
+        <v>51.39</v>
+      </c>
+      <c r="H494" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="I494" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="J494" t="n">
+        <v>18.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-13 (sentiment: 28.57)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J494"/>
+  <dimension ref="A1:J495"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16242,7 +16242,7 @@
         <v>20.93</v>
       </c>
       <c r="E494" t="n">
-        <v>7.74</v>
+        <v>6.26</v>
       </c>
       <c r="F494" t="n">
         <v>0.99</v>
@@ -16254,10 +16254,42 @@
         <v>13.29</v>
       </c>
       <c r="I494" t="n">
-        <v>9.720000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J494" t="n">
-        <v>18.85</v>
+        <v>16.57</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="n">
+        <v>46308.66666666666</v>
+      </c>
+      <c r="B495" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="C495" t="n">
+        <v>40.19</v>
+      </c>
+      <c r="D495" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="E495" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="F495" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="G495" t="n">
+        <v>51.79</v>
+      </c>
+      <c r="H495" t="n">
+        <v>58.53</v>
+      </c>
+      <c r="I495" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J495" t="n">
+        <v>28.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-14 (sentiment: 13.99)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J495"/>
+  <dimension ref="A1:J496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16274,7 +16274,7 @@
         <v>52.3</v>
       </c>
       <c r="E495" t="n">
-        <v>5.69</v>
+        <v>6.35</v>
       </c>
       <c r="F495" t="n">
         <v>3.77</v>
@@ -16286,10 +16286,42 @@
         <v>58.53</v>
       </c>
       <c r="I495" t="n">
-        <v>0.2</v>
+        <v>1.39</v>
       </c>
       <c r="J495" t="n">
-        <v>28.57</v>
+        <v>28.87</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="B496" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="C496" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="D496" t="n">
+        <v>17.55</v>
+      </c>
+      <c r="E496" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="F496" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G496" t="n">
+        <v>36.31</v>
+      </c>
+      <c r="H496" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="I496" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="J496" t="n">
+        <v>13.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-15 (sentiment: 0.60)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J496"/>
+  <dimension ref="A1:J497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16306,7 +16306,7 @@
         <v>17.55</v>
       </c>
       <c r="E496" t="n">
-        <v>7.61</v>
+        <v>6.34</v>
       </c>
       <c r="F496" t="n">
         <v>0.99</v>
@@ -16318,10 +16318,34 @@
         <v>8.529999999999999</v>
       </c>
       <c r="I496" t="n">
-        <v>10.12</v>
+        <v>1.39</v>
       </c>
       <c r="J496" t="n">
-        <v>13.99</v>
+        <v>11.81</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="n">
+        <v>46310.66666666666</v>
+      </c>
+      <c r="B497" t="inlineStr"/>
+      <c r="C497" t="inlineStr"/>
+      <c r="D497" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E497" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F497" t="inlineStr"/>
+      <c r="G497" t="inlineStr"/>
+      <c r="H497" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I497" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J497" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-16 (sentiment: 29.81)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J497"/>
+  <dimension ref="A1:J498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16334,7 +16334,7 @@
         <v>7.7</v>
       </c>
       <c r="E497" t="n">
-        <v>5.49</v>
+        <v>6.03</v>
       </c>
       <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr"/>
@@ -16348,6 +16348,38 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="498">
+      <c r="A498" s="2" t="n">
+        <v>46311.66666666666</v>
+      </c>
+      <c r="B498" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="C498" t="n">
+        <v>39.32</v>
+      </c>
+      <c r="D498" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="E498" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="F498" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="G498" t="n">
+        <v>48.01</v>
+      </c>
+      <c r="H498" t="n">
+        <v>66.47</v>
+      </c>
+      <c r="I498" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J498" t="n">
+        <v>29.81</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-19 (sentiment: 24.35)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J498"/>
+  <dimension ref="A1:J499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16362,7 +16362,7 @@
         <v>59.2</v>
       </c>
       <c r="E498" t="n">
-        <v>6.33</v>
+        <v>6.21</v>
       </c>
       <c r="F498" t="n">
         <v>2.99</v>
@@ -16374,10 +16374,42 @@
         <v>66.47</v>
       </c>
       <c r="I498" t="n">
-        <v>1.79</v>
+        <v>0.6</v>
       </c>
       <c r="J498" t="n">
-        <v>29.81</v>
+        <v>29.51</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="n">
+        <v>46314.66666666666</v>
+      </c>
+      <c r="B499" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C499" t="n">
+        <v>38.98</v>
+      </c>
+      <c r="D499" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="E499" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="F499" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G499" t="n">
+        <v>46.41</v>
+      </c>
+      <c r="H499" t="n">
+        <v>43.06</v>
+      </c>
+      <c r="I499" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="J499" t="n">
+        <v>24.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-20 (sentiment: 34.38)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J499"/>
+  <dimension ref="A1:J500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16394,7 +16394,7 @@
         <v>40.8</v>
       </c>
       <c r="E499" t="n">
-        <v>6.75</v>
+        <v>6.55</v>
       </c>
       <c r="F499" t="n">
         <v>1.39</v>
@@ -16406,10 +16406,42 @@
         <v>43.06</v>
       </c>
       <c r="I499" t="n">
-        <v>6.55</v>
+        <v>4.17</v>
       </c>
       <c r="J499" t="n">
-        <v>24.35</v>
+        <v>23.76</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="n">
+        <v>46315.66666666666</v>
+      </c>
+      <c r="B500" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="C500" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="D500" t="n">
+        <v>67.76000000000001</v>
+      </c>
+      <c r="E500" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F500" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G500" t="n">
+        <v>55.18</v>
+      </c>
+      <c r="H500" t="n">
+        <v>77.58</v>
+      </c>
+      <c r="I500" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J500" t="n">
+        <v>34.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-21 (sentiment: 24.96)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J500"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16426,7 +16426,7 @@
         <v>67.76000000000001</v>
       </c>
       <c r="E500" t="n">
-        <v>6.4</v>
+        <v>6.56</v>
       </c>
       <c r="F500" t="n">
         <v>1.39</v>
@@ -16438,10 +16438,42 @@
         <v>77.58</v>
       </c>
       <c r="I500" t="n">
-        <v>3.37</v>
+        <v>4.56</v>
       </c>
       <c r="J500" t="n">
-        <v>34.38</v>
+        <v>34.68</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="n">
+        <v>46316.66666666666</v>
+      </c>
+      <c r="B501" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="C501" t="n">
+        <v>41</v>
+      </c>
+      <c r="D501" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="E501" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G501" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="H501" t="n">
+        <v>36.71</v>
+      </c>
+      <c r="I501" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="J501" t="n">
+        <v>24.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-22 (sentiment: 14.84)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J501"/>
+  <dimension ref="A1:J502"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16458,7 +16458,7 @@
         <v>35.53</v>
       </c>
       <c r="E501" t="n">
-        <v>6.58</v>
+        <v>6.38</v>
       </c>
       <c r="F501" t="n">
         <v>0.2</v>
@@ -16470,10 +16470,42 @@
         <v>36.71</v>
       </c>
       <c r="I501" t="n">
-        <v>5.75</v>
+        <v>2.98</v>
       </c>
       <c r="J501" t="n">
-        <v>24.96</v>
+        <v>24.26</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="n">
+        <v>46317.66666666666</v>
+      </c>
+      <c r="B502" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="C502" t="n">
+        <v>40.47</v>
+      </c>
+      <c r="D502" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="E502" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="F502" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="G502" t="n">
+        <v>53.59</v>
+      </c>
+      <c r="H502" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="I502" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J502" t="n">
+        <v>14.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-23 (sentiment: 47.62)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J502"/>
+  <dimension ref="A1:J503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16490,7 +16490,7 @@
         <v>9.59</v>
       </c>
       <c r="E502" t="n">
-        <v>6.03</v>
+        <v>6.09</v>
       </c>
       <c r="F502" t="n">
         <v>2.99</v>
@@ -16502,10 +16502,34 @@
         <v>2.58</v>
       </c>
       <c r="I502" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J502" t="n">
+        <v>14.94</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="n">
+        <v>46318.66666666666</v>
+      </c>
+      <c r="B503" t="inlineStr"/>
+      <c r="C503" t="inlineStr"/>
+      <c r="D503" t="n">
+        <v>81.15000000000001</v>
+      </c>
+      <c r="E503" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="F503" t="inlineStr"/>
+      <c r="G503" t="inlineStr"/>
+      <c r="H503" t="n">
+        <v>95.04000000000001</v>
+      </c>
+      <c r="I503" t="n">
         <v>0.2</v>
       </c>
-      <c r="J502" t="n">
-        <v>14.84</v>
+      <c r="J503" t="n">
+        <v>47.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-23 (sentiment: 48.71)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -16512,16 +16512,24 @@
       <c r="A503" s="2" t="n">
         <v>46318.66666666666</v>
       </c>
-      <c r="B503" t="inlineStr"/>
-      <c r="C503" t="inlineStr"/>
+      <c r="B503" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="C503" t="n">
+        <v>41.93</v>
+      </c>
       <c r="D503" t="n">
         <v>81.15000000000001</v>
       </c>
       <c r="E503" t="n">
         <v>4.72</v>
       </c>
-      <c r="F503" t="inlineStr"/>
-      <c r="G503" t="inlineStr"/>
+      <c r="F503" t="n">
+        <v>37.65</v>
+      </c>
+      <c r="G503" t="n">
+        <v>61.95</v>
+      </c>
       <c r="H503" t="n">
         <v>95.04000000000001</v>
       </c>
@@ -16529,7 +16537,7 @@
         <v>0.2</v>
       </c>
       <c r="J503" t="n">
-        <v>47.62</v>
+        <v>48.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-26 (sentiment: 27.98)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J503"/>
+  <dimension ref="A1:J504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16522,7 +16522,7 @@
         <v>81.15000000000001</v>
       </c>
       <c r="E503" t="n">
-        <v>4.72</v>
+        <v>6.21</v>
       </c>
       <c r="F503" t="n">
         <v>37.65</v>
@@ -16534,10 +16534,34 @@
         <v>95.04000000000001</v>
       </c>
       <c r="I503" t="n">
-        <v>0.2</v>
+        <v>1.39</v>
       </c>
       <c r="J503" t="n">
-        <v>48.71</v>
+        <v>49.01</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="n">
+        <v>46321.66666666666</v>
+      </c>
+      <c r="B504" t="inlineStr"/>
+      <c r="C504" t="inlineStr"/>
+      <c r="D504" t="n">
+        <v>40.39</v>
+      </c>
+      <c r="E504" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
+      <c r="H504" t="n">
+        <v>42.66</v>
+      </c>
+      <c r="I504" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="J504" t="n">
+        <v>27.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-27 (sentiment: 16.12)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J504"/>
+  <dimension ref="A1:J505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16544,24 +16544,64 @@
       <c r="A504" s="2" t="n">
         <v>46321.66666666666</v>
       </c>
-      <c r="B504" t="inlineStr"/>
-      <c r="C504" t="inlineStr"/>
+      <c r="B504" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="C504" t="n">
+        <v>41.33</v>
+      </c>
       <c r="D504" t="n">
         <v>40.39</v>
       </c>
       <c r="E504" t="n">
-        <v>7.59</v>
-      </c>
-      <c r="F504" t="inlineStr"/>
-      <c r="G504" t="inlineStr"/>
+        <v>6.18</v>
+      </c>
+      <c r="F504" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="G504" t="n">
+        <v>59.56</v>
+      </c>
       <c r="H504" t="n">
         <v>42.66</v>
       </c>
       <c r="I504" t="n">
-        <v>13.29</v>
+        <v>0.99</v>
       </c>
       <c r="J504" t="n">
-        <v>27.98</v>
+        <v>26.85</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="n">
+        <v>46322.66666666666</v>
+      </c>
+      <c r="B505" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="C505" t="n">
+        <v>39.33</v>
+      </c>
+      <c r="D505" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="E505" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="F505" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="G505" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="H505" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="I505" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="J505" t="n">
+        <v>16.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-28 (sentiment: 38.56)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J505"/>
+  <dimension ref="A1:J506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16586,7 +16586,7 @@
         <v>10.87</v>
       </c>
       <c r="E505" t="n">
-        <v>6.83</v>
+        <v>6.14</v>
       </c>
       <c r="F505" t="n">
         <v>2.59</v>
@@ -16598,10 +16598,42 @@
         <v>3.37</v>
       </c>
       <c r="I505" t="n">
-        <v>9.720000000000001</v>
+        <v>0.99</v>
       </c>
       <c r="J505" t="n">
-        <v>16.12</v>
+        <v>13.94</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="n">
+        <v>46323.66666666666</v>
+      </c>
+      <c r="B506" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="C506" t="n">
+        <v>42.08</v>
+      </c>
+      <c r="D506" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="E506" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="F506" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="G506" t="n">
+        <v>61.95</v>
+      </c>
+      <c r="H506" t="n">
+        <v>86.31</v>
+      </c>
+      <c r="I506" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J506" t="n">
+        <v>38.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-29 (sentiment: 9.13)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J506"/>
+  <dimension ref="A1:J507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16618,7 +16618,7 @@
         <v>74.55</v>
       </c>
       <c r="E506" t="n">
-        <v>5.44</v>
+        <v>6.65</v>
       </c>
       <c r="F506" t="n">
         <v>5.78</v>
@@ -16630,10 +16630,34 @@
         <v>86.31</v>
       </c>
       <c r="I506" t="n">
-        <v>0.2</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="J506" t="n">
-        <v>38.56</v>
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="n">
+        <v>46324.66666666666</v>
+      </c>
+      <c r="B507" t="inlineStr"/>
+      <c r="C507" t="inlineStr"/>
+      <c r="D507" t="n">
+        <v>14.01</v>
+      </c>
+      <c r="E507" t="n">
+        <v>7</v>
+      </c>
+      <c r="F507" t="inlineStr"/>
+      <c r="G507" t="inlineStr"/>
+      <c r="H507" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I507" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="J507" t="n">
+        <v>9.130000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-29 (sentiment: 19.50)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -16640,16 +16640,24 @@
       <c r="A507" s="2" t="n">
         <v>46324.66666666666</v>
       </c>
-      <c r="B507" t="inlineStr"/>
-      <c r="C507" t="inlineStr"/>
+      <c r="B507" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="C507" t="n">
+        <v>40.62</v>
+      </c>
       <c r="D507" t="n">
         <v>14.01</v>
       </c>
       <c r="E507" t="n">
         <v>7</v>
       </c>
-      <c r="F507" t="inlineStr"/>
-      <c r="G507" t="inlineStr"/>
+      <c r="F507" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="G507" t="n">
+        <v>53.98</v>
+      </c>
       <c r="H507" t="n">
         <v>6.55</v>
       </c>
@@ -16657,7 +16665,7 @@
         <v>11.71</v>
       </c>
       <c r="J507" t="n">
-        <v>9.130000000000001</v>
+        <v>19.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-30 (sentiment: 18.62)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J507"/>
+  <dimension ref="A1:J508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16650,7 +16650,7 @@
         <v>14.01</v>
       </c>
       <c r="E507" t="n">
-        <v>7</v>
+        <v>5.96</v>
       </c>
       <c r="F507" t="n">
         <v>5.78</v>
@@ -16662,10 +16662,42 @@
         <v>6.55</v>
       </c>
       <c r="I507" t="n">
-        <v>11.71</v>
+        <v>0.2</v>
       </c>
       <c r="J507" t="n">
-        <v>19.5</v>
+        <v>16.63</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="n">
+        <v>46325.66666666666</v>
+      </c>
+      <c r="B508" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="C508" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="D508" t="n">
+        <v>16</v>
+      </c>
+      <c r="E508" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="F508" t="n">
+        <v>15.74</v>
+      </c>
+      <c r="G508" t="n">
+        <v>50</v>
+      </c>
+      <c r="H508" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="I508" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J508" t="n">
+        <v>18.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>